<commit_message>
Add dedicated Micron SCA tab with customer cohorts
New 'Micron SCA' sheet (after Agreements Master) detailing Micron's 16
Strategic Customer Agreements from the FQ3'26 earnings call/slides:
- Program key terms (term, volume coverage, ~$100B min revenue, $22B deposits,
  take-or-pay, floor/ceiling pricing)
- Customer cohorts: the 4 very large + 3 medium + 9 automotive split, with
  named/inferred customers (Micron does not publicly name counterparties)
- Business-unit context (CDBU/MCBU/AEBU)
Adds 3 Micron primary sources and updates Cover contents list.

Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Memory_Agreements_Hyperscalers_Neoclouds.xlsx
+++ b/Memory_Agreements_Hyperscalers_Neoclouds.xlsx
@@ -9,12 +9,13 @@
   <sheets>
     <sheet name="Cover" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Agreements Master" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Neocloud Exposure" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Pricing Benchmarks" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="HBM Generations &amp; Cost" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Supplier Allocation" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Hyperscaler Capex" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Sources" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Micron SCA" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Neocloud Exposure" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Pricing Benchmarks" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="HBM Generations &amp; Cost" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Supplier Allocation" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Hyperscaler Capex" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Sources" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -80,6 +81,16 @@
       <sz val="10"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00833C00"/>
+      <sz val="10"/>
+    </font>
+    <font>
       <i val="1"/>
       <color rgb="001F3864"/>
       <sz val="10"/>
@@ -94,7 +105,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -133,6 +144,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00C55A11"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00548235"/>
       </patternFill>
     </fill>
@@ -163,7 +179,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -200,13 +216,22 @@
     <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="4" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -231,13 +256,13 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -605,7 +630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -749,67 +774,74 @@
         </is>
       </c>
     </row>
-    <row r="23">
+    <row r="23" ht="30" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   3. Neocloud Exposure — neocloud memory exposure (mostly indirect, via GPU allocation)</t>
+          <t xml:space="preserve">   3. Micron SCA — dedicated breakdown of Micron's 16 Strategic Customer Agreements &amp; customer cohorts</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   4. Pricing Benchmarks — DRAM/HBM/NAND contract &amp; spot pricing, QoQ moves</t>
+          <t xml:space="preserve">   4. Neocloud Exposure — neocloud memory exposure (mostly indirect, via GPU allocation)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   5. HBM Generations &amp; Cost — per-stack / per-GB economics by generation</t>
+          <t xml:space="preserve">   5. Pricing Benchmarks — DRAM/HBM/NAND contract &amp; spot pricing, QoQ moves</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   6. Supplier Allocation — LTA coverage, capacity &amp; 'sold-out' status by supplier</t>
+          <t xml:space="preserve">   6. HBM Generations &amp; Cost — per-stack / per-GB economics by generation</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   7. Hyperscaler Capex — context on AI infra spend driving demand</t>
+          <t xml:space="preserve">   7. Supplier Allocation — LTA coverage, capacity &amp; 'sold-out' status by supplier</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   8. Sources — full citation list</t>
+          <t xml:space="preserve">   8. Hyperscaler Capex — context on AI infra spend driving demand</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr"/>
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   9. Sources — full citation list</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="inlineStr">
+      <c r="A30" s="4" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>CAVEATS</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="4" t="inlineStr">
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>Many headline agreements are non-binding LOIs/MOUs or remain in negotiation; values are analyst estimates and vary with the memory cycle. Specific contract pricing is almost never disclosed — per-unit figures are market benchmarks, not contract prices. Treat all numbers as directional. Verify against primary filings before use.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="30">
+  <mergeCells count="31">
     <mergeCell ref="A9:H9"/>
     <mergeCell ref="A30:H30"/>
     <mergeCell ref="A15:H15"/>
@@ -830,6 +862,7 @@
     <mergeCell ref="A14:H14"/>
     <mergeCell ref="A5:H5"/>
     <mergeCell ref="A23:H23"/>
+    <mergeCell ref="A32:H32"/>
     <mergeCell ref="A8:H8"/>
     <mergeCell ref="A22:H22"/>
     <mergeCell ref="A17:H17"/>
@@ -2347,6 +2380,613 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>MICRON STRATEGIC CUSTOMER AGREEMENTS (SCAs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Announced Micron FQ3'26 (call/slides 24 Jun 2026). 16 SCAs across data center, consumer &amp; automotive. Customers NOT publicly named by Micron.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>A) Program at a Glance — Key Terms</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>Detail</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Total agreements signed</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>16 SCAs</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Completed in fiscal Q3 2026 (announced 24 Jun 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>End markets covered</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Data center, Consumer, Automotive</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>DRAM (incl. HBM as appropriate) + NAND</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Customer cohorts</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>4 very large + 3 medium + 9 small (auto)</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>4 hyperscale-scale; 3 mid; remainder automotive OEMs</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>Standard term</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>5 years (CY2026-CY2030)</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>Automotive agreements generally 3 years</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Volume coverage</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>~20% of Micron DRAM volume; ~1/3 (33%) of NAND volume</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Over the agreement period</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>Minimum contracted revenue</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>~$100B (14 of 16 SCAs, at floor price)</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>RPO ~$100B; actual revenue expected higher</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>Cash deposits &amp; commitments</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>~$22B ($18B cash + $4B letters of credit)</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Upfront; acts as take-or-pay fail-safe / penalty</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>Contract structure</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>Take-or-pay, binding volume, non-cancellable</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>Customer cannot walk away; deposit decrements vs purchases</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>Pricing mechanism</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Price band: ceiling @ CQ2'26 market + floor through term</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Some SCAs fixed-price or no band (market-based)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>Floor economics</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Gross margin at floor &gt; any prior-cycle peak</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>Prior peak GM ~62%; recent GM ~85%</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>Revenue under SCAs (fully executed)</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>~50%+ of total company revenue</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>~40% at fixed price or ceiling at/near current market</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>Next-12-month RPO (Q3-signed)</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>~$1.8B</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>Full NTM breakdown to be disclosed from Q4</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>Capex response</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Raised toward ~$27B to expand capacity</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>$100B Clay, NY complex; volume ~FY2028</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>B) Customer Cohorts — the 4 / 3 / 9 split (customers not named by Micron)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>Cohort</t>
+        </is>
+      </c>
+      <c r="B22" s="15" t="inlineStr">
+        <is>
+          <t># Agreements</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="inlineStr">
+        <is>
+          <t>End Market</t>
+        </is>
+      </c>
+      <c r="D22" s="15" t="inlineStr">
+        <is>
+          <t>Term</t>
+        </is>
+      </c>
+      <c r="E22" s="15" t="inlineStr">
+        <is>
+          <t>Products</t>
+        </is>
+      </c>
+      <c r="F22" s="15" t="inlineStr">
+        <is>
+          <t>Pricing Structure</t>
+        </is>
+      </c>
+      <c r="G22" s="15" t="inlineStr">
+        <is>
+          <t>Named / Inferred Customers</t>
+        </is>
+      </c>
+      <c r="H22" s="15" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>Very large (hyperscale)</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>Data center</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>5 yrs (2026-2030)</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>DRAM incl. HBM (HBM3E/HBM4), NAND/eSSD</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>Price band: ceiling @ CQ2'26 + floor; some fixed</t>
+        </is>
+      </c>
+      <c r="G23" s="9" t="inlineStr">
+        <is>
+          <t>Not named. Understood to be leading hyperscalers/AI-infra buyers. Micron's disclosed HBM customers: NVIDIA (HBM4 for Vera Rubin) &amp; AMD.</t>
+        </is>
+      </c>
+      <c r="H23" s="9" t="inlineStr">
+        <is>
+          <t>Bulk of the ~$100B minimum revenue and the $22B deposits.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>Medium-sized</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>Data center / Consumer</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>Multi-year (3-5 yrs)</t>
+        </is>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>DRAM, NAND</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>Mix of price bands / fixed</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="inlineStr">
+        <is>
+          <t>Not named. Span data center and consumer electronics OEMs.</t>
+        </is>
+      </c>
+      <c r="H24" s="11" t="inlineStr">
+        <is>
+          <t>Mid-tier of contracted revenue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>Small (automotive)</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>Automotive &amp; Embedded</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>3 yrs</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="inlineStr">
+        <is>
+          <t>Auto-grade DRAM &amp; NAND</t>
+        </is>
+      </c>
+      <c r="F25" s="9" t="inlineStr">
+        <is>
+          <t>Smaller volume; market-based</t>
+        </is>
+      </c>
+      <c r="G25" s="9" t="inlineStr">
+        <is>
+          <t>Not named. Automotive OEMs / Tier-1 suppliers.</t>
+        </is>
+      </c>
+      <c r="H25" s="9" t="inlineStr">
+        <is>
+          <t>Reflects Micron's long-term commitment to the auto segment (AEBU).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="16" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B26" s="16" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="C26" s="16" t="inlineStr">
+        <is>
+          <t>DC + Consumer + Auto</t>
+        </is>
+      </c>
+      <c r="D26" s="16" t="inlineStr">
+        <is>
+          <t>3-5 yrs</t>
+        </is>
+      </c>
+      <c r="E26" s="16" t="inlineStr">
+        <is>
+          <t>DRAM (incl. HBM) + NAND</t>
+        </is>
+      </c>
+      <c r="F26" s="16" t="inlineStr">
+        <is>
+          <t>Take-or-pay; floor+ceiling bands</t>
+        </is>
+      </c>
+      <c r="G26" s="16" t="inlineStr">
+        <is>
+          <t>4 disclosed cohorts; specific names withheld</t>
+        </is>
+      </c>
+      <c r="H26" s="16" t="inlineStr">
+        <is>
+          <t>~50%+ of company revenue when fully executed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="14" t="inlineStr">
+        <is>
+          <t>C) Micron Business Units (FQ3'26 reporting segments)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="15" t="inlineStr">
+        <is>
+          <t>Business Unit</t>
+        </is>
+      </c>
+      <c r="B29" s="15" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C29" s="15" t="inlineStr">
+        <is>
+          <t>Scope</t>
+        </is>
+      </c>
+      <c r="D29" s="15" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>Core Data Center</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>CDBU</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>HBM, server DRAM, data-center SSD</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>Primary beneficiary of large hyperscale SCAs</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>Mobile &amp; Client</t>
+        </is>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>MCBU</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="inlineStr">
+        <is>
+          <t>Mobile/PC DRAM (LPDDR), client SSD</t>
+        </is>
+      </c>
+      <c r="D31" s="11" t="inlineStr">
+        <is>
+          <t>Consumer-segment SCAs</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t>Automotive &amp; Embedded</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>AEBU</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>Auto-grade DRAM/NAND, embedded</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t>9 smaller 3-yr SCAs; rev ~$4.6B, ~79% GM</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="70" customHeight="1">
+      <c r="A34" s="17" t="inlineStr">
+        <is>
+          <t>IMPORTANT: Micron did NOT publicly name any SCA counterparty. The customer identities above are cohort-level disclosures from the FQ3'26 call/slides plus reasonable inference (e.g., Micron's publicly disclosed HBM customers are NVIDIA and AMD). Do not treat inferred names as confirmed contract counterparties. Figures are at FLOOR price — actual realized revenue is expected to be higher. Source: Micron FQ3 FY2026 earnings call transcript &amp; slide deck, 24 Jun 2026 (stockanalysis.com; Micron IR slides via Fortune/Quartr); Investing.com; WCCFTech; Seoul Economic Daily.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A34:H34"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2377,52 +3017,52 @@
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="14" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>Neocloud</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>Tier</t>
         </is>
       </c>
-      <c r="C4" s="14" t="inlineStr">
+      <c r="C4" s="18" t="inlineStr">
         <is>
           <t>HQ / Region</t>
         </is>
       </c>
-      <c r="D4" s="14" t="inlineStr">
+      <c r="D4" s="18" t="inlineStr">
         <is>
           <t>Anchor Customers</t>
         </is>
       </c>
-      <c r="E4" s="14" t="inlineStr">
+      <c r="E4" s="18" t="inlineStr">
         <is>
           <t>Contracted Backlog (RPO)</t>
         </is>
       </c>
-      <c r="F4" s="14" t="inlineStr">
+      <c r="F4" s="18" t="inlineStr">
         <is>
           <t>Contracted Power</t>
         </is>
       </c>
-      <c r="G4" s="14" t="inlineStr">
+      <c r="G4" s="18" t="inlineStr">
         <is>
           <t>GPU Fleet / Orders</t>
         </is>
       </c>
-      <c r="H4" s="14" t="inlineStr">
+      <c r="H4" s="18" t="inlineStr">
         <is>
           <t>NVIDIA Relationship</t>
         </is>
       </c>
-      <c r="I4" s="14" t="inlineStr">
+      <c r="I4" s="18" t="inlineStr">
         <is>
           <t>Memory Sourcing Model</t>
         </is>
       </c>
-      <c r="J4" s="14" t="inlineStr">
+      <c r="J4" s="18" t="inlineStr">
         <is>
           <t>Notes &amp; Source</t>
         </is>
@@ -2741,7 +3381,7 @@
       </c>
     </row>
     <row r="12" ht="60" customHeight="1">
-      <c r="A12" s="15" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>KEY POINT: Neoclouds are memory price-TAKERS, not direct contract counterparties. Their HBM exposure is bundled inside Nvidia GPU systems (e.g., a Vera Rubin NVL72 rack carries ~20.7 TB of HBM4). Rising HBM4 prices ($500-600+/stack; Bernstein sees $53/GB by 2027) inflate Nvidia system prices, which flow into neocloud capex and ultimately GPU rental rates. Allocation priority (via Nvidia equity/partnership) is the real lever.</t>
         </is>
@@ -2757,7 +3397,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2789,7 +3429,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="16" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>A) Contract Price Moves (QoQ %) — the 2025-2026 surge</t>
         </is>
@@ -3052,34 +3692,34 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="inlineStr">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>B) Reference Unit Prices (mid-2026, TrendForce session/contract data)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="14" t="inlineStr">
+      <c r="A16" s="18" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B16" s="14" t="inlineStr">
+      <c r="B16" s="18" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="C16" s="14" t="inlineStr">
+      <c r="C16" s="18" t="inlineStr">
         <is>
           <t>Price (USD)</t>
         </is>
       </c>
-      <c r="D16" s="14" t="inlineStr">
+      <c r="D16" s="18" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="E16" s="14" t="inlineStr">
+      <c r="E16" s="18" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
@@ -3096,7 +3736,7 @@
           <t>DRAM chip contract</t>
         </is>
       </c>
-      <c r="C17" s="17" t="n">
+      <c r="C17" s="20" t="n">
         <v>46.83</v>
       </c>
       <c r="D17" s="9" t="inlineStr">
@@ -3121,7 +3761,7 @@
           <t>DRAM chip</t>
         </is>
       </c>
-      <c r="C18" s="18" t="n">
+      <c r="C18" s="21" t="n">
         <v>23.5</v>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -3146,7 +3786,7 @@
           <t>DRAM chip contract</t>
         </is>
       </c>
-      <c r="C19" s="17" t="n">
+      <c r="C19" s="20" t="n">
         <v>73.73999999999999</v>
       </c>
       <c r="D19" s="9" t="inlineStr">
@@ -3171,7 +3811,7 @@
           <t>DRAM chip</t>
         </is>
       </c>
-      <c r="C20" s="18" t="n">
+      <c r="C20" s="21" t="n">
         <v>36</v>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -3192,7 +3832,7 @@
           <t>Module (spot)</t>
         </is>
       </c>
-      <c r="C21" s="17" t="n">
+      <c r="C21" s="20" t="n">
         <v>208.5</v>
       </c>
       <c r="D21" s="9" t="inlineStr">
@@ -3217,7 +3857,7 @@
           <t>Server module (spot)</t>
         </is>
       </c>
-      <c r="C22" s="18" t="n">
+      <c r="C22" s="21" t="n">
         <v>1335</v>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -3242,7 +3882,7 @@
           <t>Module (spot)</t>
         </is>
       </c>
-      <c r="C23" s="17" t="n">
+      <c r="C23" s="20" t="n">
         <v>149.58</v>
       </c>
       <c r="D23" s="9" t="inlineStr">
@@ -3263,7 +3903,7 @@
           <t>HBM stack</t>
         </is>
       </c>
-      <c r="C24" s="18" t="n">
+      <c r="C24" s="21" t="n">
         <v>120</v>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -3288,7 +3928,7 @@
           <t>HBM stack</t>
         </is>
       </c>
-      <c r="C25" s="17" t="n">
+      <c r="C25" s="20" t="n">
         <v>200</v>
       </c>
       <c r="D25" s="9" t="inlineStr">
@@ -3313,7 +3953,7 @@
           <t>HBM stack</t>
         </is>
       </c>
-      <c r="C26" s="18" t="n">
+      <c r="C26" s="21" t="n">
         <v>300</v>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -3338,7 +3978,7 @@
           <t>HBM stack</t>
         </is>
       </c>
-      <c r="C27" s="17" t="n">
+      <c r="C27" s="20" t="n">
         <v>500</v>
       </c>
       <c r="D27" s="9" t="inlineStr">
@@ -3361,7 +4001,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3457,10 +4097,10 @@
           <t>8-Hi</t>
         </is>
       </c>
-      <c r="E5" s="19" t="n">
+      <c r="E5" s="22" t="n">
         <v>120</v>
       </c>
-      <c r="F5" s="20" t="n">
+      <c r="F5" s="23" t="n">
         <v>7.5</v>
       </c>
       <c r="G5" s="9" t="inlineStr">
@@ -3495,10 +4135,10 @@
           <t>12-Hi</t>
         </is>
       </c>
-      <c r="E6" s="21" t="n">
+      <c r="E6" s="24" t="n">
         <v>200</v>
       </c>
-      <c r="F6" s="22" t="n">
+      <c r="F6" s="25" t="n">
         <v>8.33</v>
       </c>
       <c r="G6" s="11" t="inlineStr">
@@ -3533,10 +4173,10 @@
           <t>12-Hi</t>
         </is>
       </c>
-      <c r="E7" s="19" t="n">
+      <c r="E7" s="22" t="n">
         <v>300</v>
       </c>
-      <c r="F7" s="20" t="n">
+      <c r="F7" s="23" t="n">
         <v>8.33</v>
       </c>
       <c r="G7" s="9" t="inlineStr">
@@ -3571,10 +4211,10 @@
           <t>16-Hi</t>
         </is>
       </c>
-      <c r="E8" s="21" t="n">
+      <c r="E8" s="24" t="n">
         <v>500</v>
       </c>
-      <c r="F8" s="22" t="n">
+      <c r="F8" s="25" t="n">
         <v>10.42</v>
       </c>
       <c r="G8" s="11" t="inlineStr">
@@ -3589,29 +4229,29 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="inlineStr">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>Nvidia per-GPU / per-rack memory economics (analyst estimates)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="14" t="inlineStr">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>Platform / Config</t>
         </is>
       </c>
-      <c r="B12" s="14" t="inlineStr">
+      <c r="B12" s="18" t="inlineStr">
         <is>
           <t>HBM Content</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
+      <c r="C12" s="18" t="inlineStr">
         <is>
           <t>Memory Cost (est.)</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr">
+      <c r="D12" s="18" t="inlineStr">
         <is>
           <t>Source / Note</t>
         </is>
@@ -3714,7 +4354,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3969,56 +4609,56 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="inlineStr">
+      <c r="A12" s="14" t="inlineStr">
         <is>
           <t>LTA structure 'new normal' (industry-wide)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="inlineStr">
+      <c r="A13" s="26" t="inlineStr">
         <is>
           <t>•  Duration: 3-5 years; formats '3yr fixed + 2yr option' or '2yr fixed + 3yr option' (UBS).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="23" t="inlineStr">
+      <c r="A14" s="26" t="inlineStr">
         <is>
           <t>•  Prepayments: 10-30% of contract value (SK hynix setting ~30% down); historically &lt;5%.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="23" t="inlineStr">
+      <c r="A15" s="26" t="inlineStr">
         <is>
           <t>•  Pricing: floor (margin protection) + ceiling (~current market) price bands; part fixed slightly below market, remainder floats.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="23" t="inlineStr">
+      <c r="A16" s="26" t="inlineStr">
         <is>
           <t>•  Take-or-pay; upfront payment forfeited as penalty if buyer under-takes committed volume.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="23" t="inlineStr">
+      <c r="A17" s="26" t="inlineStr">
         <is>
           <t>•  ~60-70% of server DDR5 volume already secured via LTAs; ~20-30% of total DRAM bits and ~20% of NAND moving to LTAs (2026-27).</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="23" t="inlineStr">
+      <c r="A18" s="26" t="inlineStr">
         <is>
           <t>•  Reserved for top-tier CSPs (MSFT, Google, Amazon, Meta, Alibaba, ByteDance) + GPU vendors (Nvidia, AMD); mid-tier pushed to spot at premium.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="23" t="inlineStr">
+      <c r="A19" s="26" t="inlineStr">
         <is>
           <t>•  Big Tech (Nvidia, Google, Amazon) offering to fund supplier fabs/equipment to strengthen allocation locks.</t>
         </is>
@@ -4040,7 +4680,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4070,22 +4710,22 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="14" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>Player</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>2026 Capex / Spend (reported)</t>
         </is>
       </c>
-      <c r="C4" s="14" t="inlineStr">
+      <c r="C4" s="18" t="inlineStr">
         <is>
           <t>Memory-relevant commitments</t>
         </is>
       </c>
-      <c r="D4" s="14" t="inlineStr">
+      <c r="D4" s="18" t="inlineStr">
         <is>
           <t>Notes &amp; Source</t>
         </is>
@@ -4254,13 +4894,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4284,22 +4924,22 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="27" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B4" s="24" t="inlineStr">
+      <c r="B4" s="27" t="inlineStr">
         <is>
           <t>Source / Outlet</t>
         </is>
       </c>
-      <c r="C4" s="24" t="inlineStr">
+      <c r="C4" s="27" t="inlineStr">
         <is>
           <t>Topic</t>
         </is>
       </c>
-      <c r="D4" s="24" t="inlineStr">
+      <c r="D4" s="27" t="inlineStr">
         <is>
           <t>Reference</t>
         </is>
@@ -4319,7 +4959,7 @@
           <t>OpenAI Stargate – Samsung &amp; SK hynix LOIs, 900k wafers/mo</t>
         </is>
       </c>
-      <c r="D5" s="25" t="inlineStr">
+      <c r="D5" s="28" t="inlineStr">
         <is>
           <t>reuters.com/business/media-telecom/samsung-sk-hynix-supply-memory-chips-openais-stargate-project-2025-10-01</t>
         </is>
@@ -4339,7 +4979,7 @@
           <t>SK hynix–OpenAI LOI, HBM for Stargate</t>
         </is>
       </c>
-      <c r="D6" s="26" t="inlineStr">
+      <c r="D6" s="29" t="inlineStr">
         <is>
           <t>eng.sk.com/news/sk-group-partners-with-openai</t>
         </is>
@@ -4359,7 +4999,7 @@
           <t>SK hynix sold out DRAM/NAND/HBM thru 2026</t>
         </is>
       </c>
-      <c r="D7" s="25" t="inlineStr">
+      <c r="D7" s="28" t="inlineStr">
         <is>
           <t>notebookcheck.net</t>
         </is>
@@ -4379,7 +5019,7 @@
           <t>Nvidia–SK hynix multi-year HBM4 deal; 60-70% Vera Rubin</t>
         </is>
       </c>
-      <c r="D8" s="26" t="inlineStr">
+      <c r="D8" s="29" t="inlineStr">
         <is>
           <t>thenextweb.com/news/nvidia-locks-in-sk-hynix</t>
         </is>
@@ -4399,7 +5039,7 @@
           <t>Nvidia–SK hynix deal; DRAM +90-95% / +58-63% QoQ; HBM4 mid-$500</t>
         </is>
       </c>
-      <c r="D9" s="25" t="inlineStr">
+      <c r="D9" s="28" t="inlineStr">
         <is>
           <t>khancapitals.com/nvidia-sk-hynix-memory-deal</t>
         </is>
@@ -4419,7 +5059,7 @@
           <t>SK hynix HBM sold out ~3 yrs; LTA requests</t>
         </is>
       </c>
-      <c r="D10" s="26" t="inlineStr">
+      <c r="D10" s="29" t="inlineStr">
         <is>
           <t>en.sedaily.com</t>
         </is>
@@ -4439,7 +5079,7 @@
           <t>Micron 16 SCAs, ~$100B min rev, floor/ceiling, $22B deposits</t>
         </is>
       </c>
-      <c r="D11" s="25" t="inlineStr">
+      <c r="D11" s="28" t="inlineStr">
         <is>
           <t>techtimes.com/articles/319032</t>
         </is>
@@ -4459,7 +5099,7 @@
           <t>Micron HBM sold out 2026; ~$22B deposits</t>
         </is>
       </c>
-      <c r="D12" s="26" t="inlineStr">
+      <c r="D12" s="29" t="inlineStr">
         <is>
           <t>karsane.com</t>
         </is>
@@ -4479,7 +5119,7 @@
           <t>Micron HBM4 36GB 12-high; full Rubin suite</t>
         </is>
       </c>
-      <c r="D13" s="25" t="inlineStr">
+      <c r="D13" s="28" t="inlineStr">
         <is>
           <t>api.finexus.net ; cryptobriefing.com</t>
         </is>
@@ -4499,7 +5139,7 @@
           <t>Samsung &amp; SK hynix reset to 3-5yr LTAs</t>
         </is>
       </c>
-      <c r="D14" s="26" t="inlineStr">
+      <c r="D14" s="29" t="inlineStr">
         <is>
           <t>trendforce.com/news/2026/04/09</t>
         </is>
@@ -4519,7 +5159,7 @@
           <t>LTAs deepen; premiums; SK hynix MSFT 3yr DDR5 / Google 5yr DRAM</t>
         </is>
       </c>
-      <c r="D15" s="25" t="inlineStr">
+      <c r="D15" s="28" t="inlineStr">
         <is>
           <t>trendforce.com/news/2026/05/04</t>
         </is>
@@ -4539,7 +5179,7 @@
           <t>HBM 2027 contract prices to surge multiples</t>
         </is>
       </c>
-      <c r="D16" s="26" t="inlineStr">
+      <c r="D16" s="29" t="inlineStr">
         <is>
           <t>trendforce.com/presscenter/news/20260602-13074</t>
         </is>
@@ -4559,7 +5199,7 @@
           <t>DDR5/DDR4 contract &amp; spot unit prices</t>
         </is>
       </c>
-      <c r="D17" s="25" t="inlineStr">
+      <c r="D17" s="28" t="inlineStr">
         <is>
           <t>trendforce.com/price/dram/dram_contract</t>
         </is>
@@ -4579,7 +5219,7 @@
           <t>DDR5 contract profitability to surpass HBM3E</t>
         </is>
       </c>
-      <c r="D18" s="26" t="inlineStr">
+      <c r="D18" s="29" t="inlineStr">
         <is>
           <t>trendforce.com/presscenter/news/20251029-12758</t>
         </is>
@@ -4599,7 +5239,7 @@
           <t>Enterprise SSD +~80% QoQ; top-5 $18.46B 1Q26</t>
         </is>
       </c>
-      <c r="D19" s="25" t="inlineStr">
+      <c r="D19" s="28" t="inlineStr">
         <is>
           <t>trendforce.com/presscenter/news/20260611-13092</t>
         </is>
@@ -4619,7 +5259,7 @@
           <t>Samsung primary HBM4 for AMD MI455X + DDR5 EPYC</t>
         </is>
       </c>
-      <c r="D20" s="26" t="inlineStr">
+      <c r="D20" s="29" t="inlineStr">
         <is>
           <t>news.samsung.com/global/samsung-and-amd ; amd.com/en/newsroom</t>
         </is>
@@ -4639,7 +5279,7 @@
           <t>Samsung weighs 3-5yr deals; Samsung-AMD HBM4/DDR5</t>
         </is>
       </c>
-      <c r="D21" s="25" t="inlineStr">
+      <c r="D21" s="28" t="inlineStr">
         <is>
           <t>bloomberg.com</t>
         </is>
@@ -4659,7 +5299,7 @@
           <t>Samsung W110tr capex; HBM4 mass prod.; Tesla $16.5B foundry</t>
         </is>
       </c>
-      <c r="D22" s="26" t="inlineStr">
+      <c r="D22" s="29" t="inlineStr">
         <is>
           <t>koreaherald.com/article/10699099</t>
         </is>
@@ -4679,7 +5319,7 @@
           <t>Big Tech (Nvidia/Google/Amazon) offer to fund SK hynix fabs</t>
         </is>
       </c>
-      <c r="D23" s="25" t="inlineStr">
+      <c r="D23" s="28" t="inlineStr">
         <is>
           <t>en.sedaily.com/society/2026/05/08</t>
         </is>
@@ -4699,7 +5339,7 @@
           <t>Advance payments / LTAs; 3-5yr CSP, 3yr GPU vendors</t>
         </is>
       </c>
-      <c r="D24" s="26" t="inlineStr">
+      <c r="D24" s="29" t="inlineStr">
         <is>
           <t>asiae.co.kr/en/article/2026040109351026768</t>
         </is>
@@ -4719,7 +5359,7 @@
           <t>LTA formats; coverage 30%/20%/18% (Samsung/Micron/SK hynix)</t>
         </is>
       </c>
-      <c r="D25" s="25" t="inlineStr">
+      <c r="D25" s="28" t="inlineStr">
         <is>
           <t>mk.co.kr/en/business/12059087</t>
         </is>
@@ -4739,7 +5379,7 @@
           <t>CXMT–Tencent ~$3B server-DRAM LTA</t>
         </is>
       </c>
-      <c r="D26" s="26" t="inlineStr">
+      <c r="D26" s="29" t="inlineStr">
         <is>
           <t>biz.chosun.com ; goldsea.com</t>
         </is>
@@ -4759,7 +5399,7 @@
           <t>Kioxia NAND seller's market; LTAs thru 2028-29; QoQ table</t>
         </is>
       </c>
-      <c r="D27" s="25" t="inlineStr">
+      <c r="D27" s="28" t="inlineStr">
         <is>
           <t>dailyalpha.us ; nand-research.com</t>
         </is>
@@ -4779,7 +5419,7 @@
           <t>HBM per-stack / per-GB cost; B200 memory $2,400</t>
         </is>
       </c>
-      <c r="D28" s="26" t="inlineStr">
+      <c r="D28" s="29" t="inlineStr">
         <is>
           <t>siliconanalysts.com/data/hbm-pricing</t>
         </is>
@@ -4799,7 +5439,7 @@
           <t>HBM4 $500-600+/stack; Rubin 6+ stacks; per-GPU $3,000-3,600</t>
         </is>
       </c>
-      <c r="D29" s="25" t="inlineStr">
+      <c r="D29" s="28" t="inlineStr">
         <is>
           <t>aicerts.ai ; nextwavesinsight.com</t>
         </is>
@@ -4819,7 +5459,7 @@
           <t>Rubin NVL72 rack $7.8M-9.1M; HBM4 ~$53/GB 2027</t>
         </is>
       </c>
-      <c r="D30" s="26" t="inlineStr">
+      <c r="D30" s="29" t="inlineStr">
         <is>
           <t>wccftech.com</t>
         </is>
@@ -4839,7 +5479,7 @@
           <t>Neocloud tiers, backlog, power, Nvidia ties</t>
         </is>
       </c>
-      <c r="D31" s="25" t="inlineStr">
+      <c r="D31" s="28" t="inlineStr">
         <is>
           <t>moduledge.com/blog/neocloud ; research.frankk.site</t>
         </is>
@@ -4859,14 +5499,74 @@
           <t>MSFT/Google 3yr DRAM deals; prepayments; ~$650B capex</t>
         </is>
       </c>
-      <c r="D32" s="26" t="inlineStr">
+      <c r="D32" s="29" t="inlineStr">
         <is>
           <t>techbriefly.com ; finance.biggo.com</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="54" customHeight="1">
-      <c r="A34" s="27" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>Micron FQ3'26 earnings call transcript (2026-06-24)</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="inlineStr">
+        <is>
+          <t>16 SCAs: terms, 4/3/9 cohorts, take-or-pay, floor/ceiling</t>
+        </is>
+      </c>
+      <c r="D33" s="28" t="inlineStr">
+        <is>
+          <t>stockanalysis.com/stocks/mu/transcripts/609470-q3-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="11" t="inlineStr">
+        <is>
+          <t>Micron FQ3'26 IR slide deck (2026-06-24)</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t>SCA volume coverage, $100B min rev, $22B deposits, BU detail</t>
+        </is>
+      </c>
+      <c r="D34" s="29" t="inlineStr">
+        <is>
+          <t>Micron IR slides via Fortune/Quartr</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="9" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>Investing.com / WCCFTech / Seoul Economic Daily (2026)</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="inlineStr">
+        <is>
+          <t>SCA $100B, $18B cash + $4B LC, 14/16 deals, non-cancellable</t>
+        </is>
+      </c>
+      <c r="D35" s="28" t="inlineStr">
+        <is>
+          <t>ng.investing.com ; wccftech.com ; en.sedaily.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="54" customHeight="1">
+      <c r="A37" s="30" t="inlineStr">
         <is>
           <t>DISCLAIMER: Compiled from secondary public sources for equity-research reference. Many agreements are non-binding (LOI/MOU) or in negotiation; values are analyst estimates that move with the memory cycle. Specific contract pricing is not publicly disclosed — unit prices shown are market benchmarks. Not investment advice. Verify against primary filings before use.</t>
         </is>
@@ -4875,8 +5575,8 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A37:D37"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A34:D34"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>